<commit_message>
Curva S actualizada 2026-07-06 11:52 Chile
</commit_message>
<xml_diff>
--- a/data/50001541 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001541 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3224" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="548">
   <si>
     <t>50001541 -  XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -6181,9 +6181,11 @@
       <c r="B70" s="5">
         <v>46132.58888190972</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46209.63277412037</v>
+      </c>
       <c r="D70" s="5">
-        <v>46196.691984930556</v>
+        <v>46209.6327872338</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>232</v>
@@ -6218,8 +6220,12 @@
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
-      <c r="T70" s="6"/>
-      <c r="U70" s="6"/>
+      <c r="T70" s="6">
+        <v>1</v>
+      </c>
+      <c r="U70" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
@@ -7238,9 +7244,11 @@
       <c r="B89" s="8">
         <v>46132.58889809028</v>
       </c>
-      <c r="C89" s="9"/>
+      <c r="C89" s="8">
+        <v>46209.6327590162</v>
+      </c>
       <c r="D89" s="8">
-        <v>46203.20341778935</v>
+        <v>46209.63276071759</v>
       </c>
       <c r="E89" s="9" t="s">
         <v>269</v>
@@ -7290,8 +7298,8 @@
       <c r="T89" s="9">
         <v>1</v>
       </c>
-      <c r="U89" s="10" t="s">
-        <v>98</v>
+      <c r="U89" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -8016,9 +8024,11 @@
       <c r="B103" s="8">
         <v>46132.63157251157</v>
       </c>
-      <c r="C103" s="9"/>
+      <c r="C103" s="8">
+        <v>46209.63248238426</v>
+      </c>
       <c r="D103" s="8">
-        <v>46196.912235208336</v>
+        <v>46209.63248512732</v>
       </c>
       <c r="E103" s="9" t="s">
         <v>273</v>
@@ -8069,9 +8079,11 @@
       <c r="B104" s="5">
         <v>46132.631576643515</v>
       </c>
-      <c r="C104" s="6"/>
+      <c r="C104" s="5">
+        <v>46209.63248900463</v>
+      </c>
       <c r="D104" s="5">
-        <v>46196.91224765046</v>
+        <v>46209.63249092593</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>173</v>
@@ -8122,9 +8134,11 @@
       <c r="B105" s="8">
         <v>46132.6319078588</v>
       </c>
-      <c r="C105" s="9"/>
+      <c r="C105" s="8">
+        <v>46209.63249508102</v>
+      </c>
       <c r="D105" s="8">
-        <v>46196.91227103009</v>
+        <v>46209.63249679398</v>
       </c>
       <c r="E105" s="9" t="s">
         <v>273</v>
@@ -9248,7 +9262,7 @@
         <v>46205.49134238426</v>
       </c>
       <c r="D125" s="8">
-        <v>46205.4913437037</v>
+        <v>46209.63248880787</v>
       </c>
       <c r="E125" s="9" t="s">
         <v>173</v>
@@ -9303,7 +9317,7 @@
         <v>46205.49141931713</v>
       </c>
       <c r="D126" s="5">
-        <v>46205.49142064815</v>
+        <v>46209.63249525463</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>173</v>
@@ -9358,7 +9372,7 @@
         <v>46205.49149630787</v>
       </c>
       <c r="D127" s="8">
-        <v>46205.49149763889</v>
+        <v>46209.632502152774</v>
       </c>
       <c r="E127" s="9" t="s">
         <v>173</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-30 13:27 Chile
</commit_message>
<xml_diff>
--- a/data/50001541 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001541 - XEMORTIZ MINERA FRISCO.xlsx
@@ -2655,7 +2655,7 @@
         <v>46198.65467643518</v>
       </c>
       <c r="D10" s="5">
-        <v>46198.65469435185</v>
+        <v>46264.463179178245</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>44</v>
@@ -6297,7 +6297,7 @@
         <v>46196.69197697917</v>
       </c>
       <c r="D72" s="5">
-        <v>46260.58108960648</v>
+        <v>46264.05806130787</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>238</v>

</xml_diff>